<commit_message>
Restore the German matiere overrides as an explicit override column
The German correction sheet recorded its manual corrections by
overwriting `matiere` in place, so re-exporting silently reverted them:
the whole Willehalm cycle (Willehalm, Rennewart, Arabel, Willehalm von
Orlens, the prose Willehalm, Sibille) fell back from France to Other,
and Alpharts Tod from Other to England.

These 7 works have no storyverse-derived matiere at all (matieres empty,
matter_local = Other), so the automatic resolution cannot place them --
they need a manual assignment. Recovered by diffing the original sheet
against what the resolution formula derives, and recorded in the same
explicit `override` column French uses, so a re-export can no longer
drop them.

Verified: 01-networks now reproduces the original baseline exactly --
german France back to 20 nodes, Other 44, England 3, Heldendichtung 18.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/german_works.xlsx
+++ b/data/german_works.xlsx
@@ -500,7 +500,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="G2" t="b">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>France</t>
         </is>
       </c>
       <c r="G57" t="b">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>France</t>
         </is>
       </c>
       <c r="G71" t="b">
@@ -3371,7 +3371,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>France</t>
         </is>
       </c>
       <c r="G101" t="b">
@@ -3516,7 +3516,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>France</t>
         </is>
       </c>
       <c r="G106" t="b">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>France</t>
         </is>
       </c>
       <c r="G110" t="b">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>France</t>
         </is>
       </c>
       <c r="G116" t="b">

</xml_diff>

<commit_message>
Move remaining value-cleaning out of 01-networks into the export
load_linkage was still unquoting German work titles and title-casing
witness status at analysis time, and assign_matiere still had an
empty-string fallback. Those are preprocessing concerns: the export now
does them once, and the analysis notebook restores JSON dtypes and
nothing else.

Splitting this logic across both notebooks is what produced the original
inconsistencies -- 01-networks aliased england -> Britain while the
export kept England, and neither applied the manual corrections. With
the export owning all of it, there is one place to look.

Data files rewritten accordingly: 374 German linkage titles and 82
German work titles unquoted, status normalised to title case in both
languages. Verified unchanged: french 256/907, german 118/187, 18
Heldendichtung, no node name carries quotes, no cell fails.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/german_works.xlsx
+++ b/data/german_works.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>'Alpharts Tod'</t>
+          <t>Alpharts Tod</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -513,7 +513,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>'Bairisch-österreichisches Buch von Troja' (früher: 'Buch von Troja II')</t>
+          <t>Bairisch-österreichisches Buch von Troja' (früher: 'Buch von Troja II')</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>'Biterolf und Dietleib' ('Biterolf')</t>
+          <t>Biterolf und Dietleib' ('Biterolf')</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -581,7 +581,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>'Breslauer Apollonius'</t>
+          <t>Breslauer Apollonius</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>'Buch von Troja nach Guido de Columnis'</t>
+          <t>Buch von Troja nach Guido de Columnis</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>'Cleomades'</t>
+          <t>Cleomades</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -683,7 +683,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>'Daniel'</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>'Der Große Alexander'</t>
+          <t>Der Große Alexander</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>'Der Wunderer'</t>
+          <t>Der Wunderer</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>'Die gute Frau'</t>
+          <t>Die gute Frau</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>'Die Königin vom Brennenden See'</t>
+          <t>Die Königin vom Brennenden See</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>'Dietrichs Flucht'</t>
+          <t>Dietrichs Flucht</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>'Eckenlied'</t>
+          <t>Eckenlied</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>'Elsässisches Trojabuch'</t>
+          <t>Elsässisches Trojabuch</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>'Friedrich von Schwaben'</t>
+          <t>Friedrich von Schwaben</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>'Göttweiger Trojanerkrieg'</t>
+          <t>Göttweiger Trojanerkrieg</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>'Herzog Ernst' B</t>
+          <t>Herzog Ernst' B</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>'Herzog Ernst' D</t>
+          <t>Herzog Ernst' D</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>'Herzog Ernst' F</t>
+          <t>Herzog Ernst' F</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>'Herzog Ernst' G</t>
+          <t>Herzog Ernst' G</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>'Hildebrandslied'</t>
+          <t>Hildebrandslied</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>'Historie van Sent Reinolt'</t>
+          <t>Historie van Sent Reinolt</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>'Johann aus dem Virgiere'</t>
+          <t>Johann aus dem Virgiere</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>'Jüngeres Hildebrandslied'</t>
+          <t>Jüngeres Hildebrandslied</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>'Karl und Elegast'</t>
+          <t>Karl und Elegast</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>'Karlmeinet'-Kompilation</t>
+          <t>Karlmeinet'-Kompilation</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>'König Rother'</t>
+          <t>König Rother</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>'Kudrun'</t>
+          <t>Kudrun</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>'Lancelot'</t>
+          <t>Lancelot</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>'Laurin'</t>
+          <t>Laurin</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>'Leipziger Apollonius'</t>
+          <t>Leipziger Apollonius</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>'Lohengrin'</t>
+          <t>Lohengrin</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>'Mai und Beaflor'</t>
+          <t>Mai und Beaflor</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>'Malagis'</t>
+          <t>Malagis</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>'Morant und Galie'</t>
+          <t>Morant und Galie</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>'Münchner Oswald'</t>
+          <t>Münchner Oswald</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>'Nibelungenlied'</t>
+          <t>Nibelungenlied</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>'Ogier von Dänemark'</t>
+          <t>Ogier von Dänemark</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>'Ortnit'</t>
+          <t>Ortnit</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>'Oswald' / 'Berliner Oswald'</t>
+          <t>Oswald' / 'Berliner Oswald</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>'Pontus und Sidonia'</t>
+          <t>Pontus und Sidonia</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>'Rabenschlacht'</t>
+          <t>Rabenschlacht</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>'Rappoltsteiner Parzifal'</t>
+          <t>Rappoltsteiner Parzifal</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>'Reinfried von Braunschweig'</t>
+          <t>Reinfried von Braunschweig</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1975,7 +1975,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>'Reinolt von Montelban'</t>
+          <t>Reinolt von Montelban</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>'Rosengarten zu Worms'</t>
+          <t>Rosengarten zu Worms</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>'Salman und Morolf'</t>
+          <t>Salman und Morolf</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>'Sigenot'</t>
+          <t>Sigenot</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>'Tristan als Mönch'</t>
+          <t>Tristan als Mönch</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>'Trojanerkrieg'</t>
+          <t>Trojanerkrieg</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>'Trojanerkrieg'-Fortsetzung</t>
+          <t>Trojanerkrieg'-Fortsetzung</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>'Virginal'</t>
+          <t>Virginal</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>'Walberan'</t>
+          <t>Walberan</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>'Wiener Oswald'</t>
+          <t>Wiener Oswald</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>'Wigamur'</t>
+          <t>Wigamur</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>'Willehalm' (Prosaroman)</t>
+          <t>Willehalm' (Prosaroman)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>'Wolfdietrich'</t>
+          <t>Wolfdietrich</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2417,7 +2417,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>'Zürcher Buch vom heiligen Karl'</t>
+          <t>Zürcher Buch vom heiligen Karl</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Albrecht von Kemenaten: 'Goldemar'</t>
+          <t>Albrecht von Kemenaten: 'Goldemar</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Albrecht: 'Jüngerer Titurel'</t>
+          <t>Albrecht: 'Jüngerer Titurel</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Berthold von Holle: 'Crane'</t>
+          <t>Berthold von Holle: 'Crane</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Berthold von Holle: 'Demantin'</t>
+          <t>Berthold von Holle: 'Demantin</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Der Pleier: 'Garel von dem blühenden Tal'</t>
+          <t>Der Pleier: 'Garel von dem blühenden Tal</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Der Pleier: 'Meleranz'</t>
+          <t>Der Pleier: 'Meleranz</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Der Pleier: 'Tandareis und Flordibel'</t>
+          <t>Der Pleier: 'Tandareis und Flordibel</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Eilhart von Oberg: 'Tristrant'</t>
+          <t>Eilhart von Oberg: 'Tristrant</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Elisabeth von Nassau-Saarbrücken: 'Herpin'</t>
+          <t>Elisabeth von Nassau-Saarbrücken: 'Herpin</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Elisabeth von Nassau-Saarbrücken: 'Huge Scheppel'</t>
+          <t>Elisabeth von Nassau-Saarbrücken: 'Huge Scheppel</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Elisabeth von Nassau-Saarbrücken: 'Loher und Maller'</t>
+          <t>Elisabeth von Nassau-Saarbrücken: 'Loher und Maller</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Elisabeth von Nassau-Saarbrücken: 'Sibille'</t>
+          <t>Elisabeth von Nassau-Saarbrücken: 'Sibille</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Fleck, Konrad: 'Flore und Blanscheflur'</t>
+          <t>Fleck, Konrad: 'Flore und Blanscheflur</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2961,7 +2961,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Gottfried von Straßburg: 'Tristan'</t>
+          <t>Gottfried von Straßburg: 'Tristan</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Gutevrunt, Heinrich: 'Historia von der vorstorunge troye'</t>
+          <t>Gutevrunt, Heinrich: 'Historia von der vorstorunge troye</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Hartlieb, Johannes: 'Alexander'</t>
+          <t>Hartlieb, Johannes: 'Alexander</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3063,7 +3063,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Hartmann von Aue: 'Der arme Heinrich'</t>
+          <t>Hartmann von Aue: 'Der arme Heinrich</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3097,7 +3097,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Hartmann von Aue: 'Erec'</t>
+          <t>Hartmann von Aue: 'Erec</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Hartmann von Aue: 'Gregorius'</t>
+          <t>Hartmann von Aue: 'Gregorius</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Hartmann von Aue: 'Iwein'</t>
+          <t>Hartmann von Aue: 'Iwein</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Heinrich von dem Türlin: 'Diu Crône'</t>
+          <t>Heinrich von dem Türlin: 'Diu Crône</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Heinrich von Freiberg: 'Tristan'</t>
+          <t>Heinrich von Freiberg: 'Tristan</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Heinrich von Neustadt: 'Apollonius von Tyrland'</t>
+          <t>Heinrich von Neustadt: 'Apollonius von Tyrland</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Heinrich von Veldeke: 'Eneas'</t>
+          <t>Heinrich von Veldeke: 'Eneas</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Herbort von Fritzlar: 'Liet von Troye'</t>
+          <t>Herbort von Fritzlar: 'Liet von Troye</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Johann von Würzburg: 'Wilhelm von Österreich'</t>
+          <t>Johann von Würzburg: 'Wilhelm von Österreich</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -3403,7 +3403,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Konrad von Stoffeln: 'Gauriel von Muntabel'</t>
+          <t>Konrad von Stoffeln: 'Gauriel von Muntabel</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Konrad von Würzburg: 'Partonopier und Meliur'</t>
+          <t>Konrad von Würzburg: 'Partonopier und Meliur</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Konrad von Würzburg: 'Trojanerkrieg'</t>
+          <t>Konrad von Würzburg: 'Trojanerkrieg</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3505,7 +3505,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Mair, Hans, von Nördlingen: 'Buch von Troja'</t>
+          <t>Mair, Hans, von Nördlingen: 'Buch von Troja</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Meister Wichwolt [früher: Babiloth]: 'Cronica Allexandri des grossen konigs'</t>
+          <t>Meister Wichwolt [früher: Babiloth]: 'Cronica Allexandri des grossen konigs</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Otte: 'Eraclius'</t>
+          <t>Otte: 'Eraclius</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -3607,7 +3607,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Otto II. von Freising: 'Barlaam und Josaphat'</t>
+          <t>Otto II. von Freising: 'Barlaam und Josaphat</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -3641,7 +3641,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Pfaffe Konrad: 'Rolandslied'</t>
+          <t>Pfaffe Konrad: 'Rolandslied</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Pfaffe Lambrecht: 'Alexanderlied'</t>
+          <t>Pfaffe Lambrecht: 'Alexanderlied</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3709,7 +3709,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>'Der Mantel'</t>
+          <t>Der Mantel</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Rudolf von Ems: 'Alexander'</t>
+          <t>Rudolf von Ems: 'Alexander</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Rudolf von Ems: 'Barlaam und Josaphat'</t>
+          <t>Rudolf von Ems: 'Barlaam und Josaphat</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Rudolf von Ems: 'Der guote Gêrhart'</t>
+          <t>Rudolf von Ems: 'Der guote Gêrhart</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Rudolf von Ems: 'Willehalm von Orlens'</t>
+          <t>Rudolf von Ems: 'Willehalm von Orlens</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Seifrit: 'Alexander'</t>
+          <t>Seifrit: 'Alexander</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Steinhöwel, Heinrich: 'Apollonius'</t>
+          <t>Steinhöwel, Heinrich: 'Apollonius</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Stricker: 'Karl der Große'</t>
+          <t>Stricker: 'Karl der Große</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4015,7 +4015,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Ulrich von dem Türlin: 'Arabel'</t>
+          <t>Ulrich von dem Türlin: 'Arabel</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -4049,7 +4049,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Ulrich von Etzenbach: 'Alexander'</t>
+          <t>Ulrich von Etzenbach: 'Alexander</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Ulrich von Etzenbach: 'Alexander-Anhang'</t>
+          <t>Ulrich von Etzenbach: 'Alexander-Anhang</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Ulrich von Etzenbach: 'Wilhelm von Wenden'</t>
+          <t>Ulrich von Etzenbach: 'Wilhelm von Wenden</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -4151,7 +4151,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Ulrich von Türheim: 'Rennewart'</t>
+          <t>Ulrich von Türheim: 'Rennewart</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Ulrich von Türheim: 'Tristan'</t>
+          <t>Ulrich von Türheim: 'Tristan</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Ulrich von Zatzikhoven: 'Lanzelet'</t>
+          <t>Ulrich von Zatzikhoven: 'Lanzelet</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Wirnt von Grafenberg: 'Wigalois'</t>
+          <t>Wirnt von Grafenberg: 'Wigalois</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -4287,7 +4287,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Wolfram von Eschenbach: 'Parzival'</t>
+          <t>Wolfram von Eschenbach: 'Parzival</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -4321,7 +4321,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Wolfram von Eschenbach: 'Titurel'</t>
+          <t>Wolfram von Eschenbach: 'Titurel</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -4355,7 +4355,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Wolfram von Eschenbach: 'Willehalm'</t>
+          <t>Wolfram von Eschenbach: 'Willehalm</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -4389,7 +4389,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>'Abor und das Meerweib'</t>
+          <t>Abor und das Meerweib</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -4423,7 +4423,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>'Ainune'</t>
+          <t>Ainune</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>'Alischanz'</t>
+          <t>Alischanz</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>'Athis und Prophilias'</t>
+          <t>Athis und Prophilias</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -4525,7 +4525,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>'Dietrich und Fasold'</t>
+          <t>Dietrich und Fasold</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -4559,7 +4559,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>'Dietrich und Wenezlan'</t>
+          <t>Dietrich und Wenezlan</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -4593,7 +4593,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>'Edolanz'</t>
+          <t>Edolanz</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>'Graf Rudolf'</t>
+          <t>Graf Rudolf</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>'Herzog Ernst' A</t>
+          <t>Herzog Ernst' A</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>'Herzog Ernst' Kl</t>
+          <t>Herzog Ernst' Kl</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -4729,7 +4729,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>'Hürnen Seyfrid'</t>
+          <t>Hürnen Seyfrid</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>'Karl und Galie'</t>
+          <t>Karl und Galie</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>'Linzer Oswald'</t>
+          <t>Linzer Oswald</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>'Manuel und Amande'</t>
+          <t>Manuel und Amande</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -4865,7 +4865,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>'Mitteldeutscher Erec'</t>
+          <t>Mitteldeutscher Erec</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>'Niederfränkischer Tristan'</t>
+          <t>Niederfränkischer Tristan</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>'Ospinel'</t>
+          <t>Ospinel</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -4967,7 +4967,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>'Parcheval'</t>
+          <t>Parcheval</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>'Segremors'</t>
+          <t>Segremors</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -5035,7 +5035,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>'Trierer Floyris'</t>
+          <t>Trierer Floyris</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -5069,7 +5069,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>'Waldecker (Marburger) Alexander'</t>
+          <t>Waldecker (Marburger) Alexander</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -5103,7 +5103,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>'Walther und Hildegund'</t>
+          <t>Walther und Hildegund</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Berthold von Holle: 'Darifant'</t>
+          <t>Berthold von Holle: 'Darifant</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Dietrich von Hopfgarten: 'Wigelis'</t>
+          <t>Dietrich von Hopfgarten: 'Wigelis</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Hans von Bühel: 'Die Königstochter von Frankreich'</t>
+          <t>Hans von Bühel: 'Die Königstochter von Frankreich</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -5239,7 +5239,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Ulrich von Türheim: 'Kliges'</t>
+          <t>Ulrich von Türheim: 'Kliges</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>'Orendel' ('Der Graue Rock')</t>
+          <t>Orendel' ('Der Graue Rock')</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">

</xml_diff>